<commit_message>
Production Files Rev02 - second try :)
</commit_message>
<xml_diff>
--- a/Strommessplatine/Project Outputs for Strommessplatine/Rev02/BOM_JLC/BOM_JLC_Strommessplatine_Default_Rev02.xlsx
+++ b/Strommessplatine/Project Outputs for Strommessplatine/Rev02/BOM_JLC/BOM_JLC_Strommessplatine_Default_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\uz_per_external_current_sensing\Strommessplatine\Project Outputs for Strommessplatine\Rev02\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C3EBA3A-AD18-409E-907C-8B96C5FF2EC8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C9C3077-497C-4A85-BE41-DE7E32B0D016}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18460" windowHeight="9400" xr2:uid="{0D09DFE8-AEEA-4970-B309-3FB0D2072504}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18700" windowHeight="9730" xr2:uid="{C68E8B44-3F05-48E4-87D9-618E64152BD6}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_Strommessplatine_Defaul" sheetId="1" r:id="rId1"/>
@@ -793,7 +793,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B37FC920-8AE7-49D7-9F6A-145299376DE6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8D8E6DD-5359-4FAD-8BD7-A258FED75E11}">
   <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>